<commit_message>
fix: resolve Excel formula error by replacing Python exponentiation ** with Excel caret ^
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_tco_estimator.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_tco_estimator.xlsx
@@ -998,11 +998,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="142" customWidth="1" min="2" max="2"/>
-    <col width="142" customWidth="1" min="3" max="3"/>
-    <col width="142" customWidth="1" min="4" max="4"/>
-    <col width="142" customWidth="1" min="5" max="5"/>
-    <col width="142" customWidth="1" min="6" max="6"/>
+    <col width="141" customWidth="1" min="2" max="2"/>
+    <col width="141" customWidth="1" min="3" max="3"/>
+    <col width="141" customWidth="1" min="4" max="4"/>
+    <col width="141" customWidth="1" min="5" max="5"/>
+    <col width="141" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -1205,23 +1205,23 @@
         </is>
       </c>
       <c r="B13" s="17">
-        <f>B11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)**(1-1)</f>
+        <f>B11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)^(1-1)</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>C11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)**(2-1)</f>
+        <f>C11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)^(2-1)</f>
         <v/>
       </c>
       <c r="D13" s="17">
-        <f>D11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)**(3-1)</f>
+        <f>D11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)^(3-1)</f>
         <v/>
       </c>
       <c r="E13" s="17">
-        <f>E11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)**(4-1)</f>
+        <f>E11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)^(4-1)</f>
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>F11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)**(5-1)</f>
+        <f>F11*(('💡 說明與變數設定'!$B$22*'💡 說明與變數設定'!$B$20/1000)+('💡 說明與變數設定'!$B$23*'💡 說明與變數設定'!$B$21/1000))*'💡 說明與變數設定'!$B$18*(1+'💡 說明與變數設定'!$B$15)^(5-1)</f>
         <v/>
       </c>
     </row>

</xml_diff>